<commit_message>
Sprint6 (Day45): complete Day 45 final sign-off, acceptance checklist PDF, and deliverables archive
</commit_message>
<xml_diff>
--- a/output/final_deliverables/peer_comparison.xlsx
+++ b/output/final_deliverables/peer_comparison.xlsx
@@ -850,7 +850,7 @@
         <v>45133</v>
       </c>
       <c r="M3" t="n">
-        <v>2.18</v>
+        <v>4.06</v>
       </c>
       <c r="N3" t="n">
         <v>75.81</v>
@@ -1395,7 +1395,7 @@
         <v>-11245</v>
       </c>
       <c r="M8" t="n">
-        <v>1.39</v>
+        <v>1.11</v>
       </c>
       <c r="N8" t="n">
         <v>-45.18</v>
@@ -1834,7 +1834,7 @@
         <v>-29445</v>
       </c>
       <c r="M2" t="n">
-        <v>1.42</v>
+        <v>1.94</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
@@ -1931,7 +1931,7 @@
         <v>13296</v>
       </c>
       <c r="M3" t="n">
-        <v>4.81</v>
+        <v>6.2</v>
       </c>
       <c r="N3" t="n">
         <v>28.81</v>
@@ -2042,7 +2042,7 @@
         <v>-7559</v>
       </c>
       <c r="M4" t="n">
-        <v>6.5</v>
+        <v>4.35</v>
       </c>
       <c r="N4" t="n">
         <v>-17.03</v>
@@ -2149,7 +2149,7 @@
         <v>-7559</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>4.81</v>
+        <v>4.35</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>5.889999999999999</v>
@@ -2243,7 +2243,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
@@ -2487,7 +2487,7 @@
         <v>9789</v>
       </c>
       <c r="M2" t="n">
-        <v>3.34</v>
+        <v>5.16</v>
       </c>
       <c r="N2" t="n">
         <v>5.1</v>
@@ -2598,7 +2598,7 @@
         <v>-2336</v>
       </c>
       <c r="M3" t="n">
-        <v>-1.99</v>
+        <v>1.94</v>
       </c>
       <c r="N3" t="n">
         <v>-22.9</v>
@@ -2701,7 +2701,7 @@
         <v>-2389</v>
       </c>
       <c r="M4" t="n">
-        <v>1.93</v>
+        <v>3.4</v>
       </c>
       <c r="N4" t="n">
         <v>-8.48</v>
@@ -2813,7 +2813,7 @@
         <v>6048</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>-0.13</v>
+        <v>4.74</v>
       </c>
       <c r="N5" s="5" t="n">
         <v>27.18</v>
@@ -2908,7 +2908,7 @@
         <v>1856</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>0.8999999999999999</v>
+        <v>4.07</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>-1.69</v>
@@ -4453,7 +4453,7 @@
         <v>26</v>
       </c>
       <c r="M7" t="n">
-        <v>0.89</v>
+        <v>1.25</v>
       </c>
       <c r="N7" t="n">
         <v>1.14</v>
@@ -4564,7 +4564,7 @@
         <v>-1365</v>
       </c>
       <c r="M8" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.09</v>
       </c>
       <c r="N8" t="n">
         <v>-46.16</v>
@@ -4659,7 +4659,7 @@
         <v>2938</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1.04</v>
+        <v>1.06</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>43.42</v>
@@ -5642,7 +5642,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
@@ -6103,7 +6103,9 @@
       <c r="L4" t="n">
         <v>-2893</v>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>5.22</v>
+      </c>
       <c r="N4" t="n">
         <v>-2.87</v>
       </c>
@@ -6320,7 +6322,7 @@
         <v>-997</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>8.91</v>
+        <v>7.065</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>-1.38</v>
@@ -6881,7 +6883,7 @@
         <v>39635</v>
       </c>
       <c r="M4" t="n">
-        <v>2.05</v>
+        <v>2.59</v>
       </c>
       <c r="N4" t="n">
         <v>52.4</v>
@@ -7211,7 +7213,7 @@
         <v>39635</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2.05</v>
+        <v>2.22</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>40.9</v>
@@ -8439,7 +8441,7 @@
         <v>17651</v>
       </c>
       <c r="M2" t="n">
-        <v>-1.03</v>
+        <v>3.72</v>
       </c>
       <c r="N2" t="n">
         <v>96.83</v>
@@ -9099,7 +9101,7 @@
         <v>-13347</v>
       </c>
       <c r="M8" t="n">
-        <v>-1.1</v>
+        <v>7.19</v>
       </c>
       <c r="N8" t="n">
         <v>-182.39</v>
@@ -9198,7 +9200,7 @@
         <v>3569</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1.91</v>
+        <v>3.72</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>20.18</v>

</xml_diff>